<commit_message>
Standard calibration + federated intercept recalibration
- Calibration slope/intercept now use the standard regression-based definitions (Cox calibration slope; calibration-in-the-large via an offset logistic model) instead of a binned reliability-curve fit.
- Add a federated intercept-recalibration step after FedAvg that removes the calibration-in-the-large offset, sharing only aggregate scalars.
- Figure 4 PCA now uses the full model parameters (slopes + intercept) and includes the recalibrated FL model.
- Convergence figure/summary report the recalibration step and total wall-clock time.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/PCA.xlsx
+++ b/outputs/PCA.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,10 +480,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.2335997958387242</v>
+        <v>3.809135726130791</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4001069679386829</v>
+        <v>1.806443849721656</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -496,10 +496,10 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.2466633157753654</v>
+        <v>3.78531183099556</v>
       </c>
       <c r="I2" t="n">
-        <v>0.38991307920743</v>
+        <v>1.431244079353054</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -512,10 +512,10 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>0.2416400326747687</v>
+        <v>3.767167895003664</v>
       </c>
       <c r="N2" t="n">
-        <v>0.3981391199909893</v>
+        <v>1.642206483914608</v>
       </c>
     </row>
     <row r="3">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.03991187426225484</v>
+        <v>-0.8990676035591187</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.107587877628387</v>
+        <v>-0.5945389961139496</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.0390901866522512</v>
+        <v>-0.8658430900740995</v>
       </c>
       <c r="I3" t="n">
-        <v>-0.1015298645054449</v>
+        <v>-0.3862191715429833</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>0.04219427587540745</v>
+        <v>-0.8598931807648466</v>
       </c>
       <c r="N3" t="n">
-        <v>-0.1094199288336712</v>
+        <v>-0.5193677382601622</v>
       </c>
     </row>
     <row r="4">
@@ -580,10 +580,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-0.1405591847645656</v>
+        <v>-1.084264594877617</v>
       </c>
       <c r="D4" t="n">
-        <v>0.02130476098091414</v>
+        <v>0.09838513048892121</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -596,10 +596,10 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>-0.136610853366873</v>
+        <v>-1.077396816323406</v>
       </c>
       <c r="I4" t="n">
-        <v>0.02287122930603581</v>
+        <v>-0.02369047126554166</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -612,10 +612,10 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>-0.1350621434562185</v>
+        <v>-1.070118543415887</v>
       </c>
       <c r="N4" t="n">
-        <v>0.02069603472850719</v>
+        <v>0.014317461487131</v>
       </c>
     </row>
     <row r="5">
@@ -630,10 +630,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-0.007036330490856274</v>
+        <v>-0.3162962725104385</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.007580857396270506</v>
+        <v>-0.1097125770120243</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -646,10 +646,10 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>-0.003804613950110903</v>
+        <v>-0.2738090121156291</v>
       </c>
       <c r="I5" t="n">
-        <v>-0.01216537866009891</v>
+        <v>-0.08986277316627361</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -662,10 +662,10 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>-0.004525878748340832</v>
+        <v>-0.2912335476928489</v>
       </c>
       <c r="N5" t="n">
-        <v>-0.009883525963478296</v>
+        <v>-0.0953496938336722</v>
       </c>
     </row>
     <row r="6">
@@ -680,10 +680,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.1342350051275184</v>
+        <v>-0.0994485205041607</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01451076262045566</v>
+        <v>1.614739473810381</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -696,10 +696,10 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.1356225793150522</v>
+        <v>-0.0516619890376381</v>
       </c>
       <c r="I6" t="n">
-        <v>0.0130666345243872</v>
+        <v>2.00011987993266</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -712,10 +712,10 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>0.1368882478594342</v>
+        <v>-0.05089276712662254</v>
       </c>
       <c r="N6" t="n">
-        <v>0.009608521988649537</v>
+        <v>1.884738229614658</v>
       </c>
     </row>
     <row r="7">
@@ -730,10 +730,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.408399768083176</v>
+        <v>-3.727985668250426</v>
       </c>
       <c r="D7" t="n">
-        <v>0.05757688130690966</v>
+        <v>1.412872494767792</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -746,10 +746,10 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>-0.4048775647322218</v>
+        <v>-3.6995568472853</v>
       </c>
       <c r="I7" t="n">
-        <v>0.06611403892444677</v>
+        <v>1.436410710900394</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -762,10 +762,10 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>-0.4051499332956596</v>
+        <v>-3.708953969313856</v>
       </c>
       <c r="N7" t="n">
-        <v>0.05647275705802065</v>
+        <v>1.388243859131896</v>
       </c>
     </row>
     <row r="8">
@@ -780,10 +780,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-0.07302535700835414</v>
+        <v>-0.5658448851754394</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1750841880511178</v>
+        <v>1.810956133910129</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -796,10 +796,10 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>-0.06998094668597706</v>
+        <v>-0.5834925729863586</v>
       </c>
       <c r="I8" t="n">
-        <v>0.180362276925103</v>
+        <v>1.715705887241277</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -812,10 +812,10 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>-0.07132478835052239</v>
+        <v>-0.595137857836369</v>
       </c>
       <c r="N8" t="n">
-        <v>0.1726996523982158</v>
+        <v>1.737310878400666</v>
       </c>
     </row>
     <row r="9">
@@ -830,10 +830,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.1717691125793171</v>
+        <v>-0.3186410881819956</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.04090826013977042</v>
+        <v>-0.9816734049708037</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -846,10 +846,10 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>-0.1703843209564558</v>
+        <v>-0.3098513411681695</v>
       </c>
       <c r="I9" t="n">
-        <v>-0.04021128692928785</v>
+        <v>-1.168988089688637</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -862,10 +862,10 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>-0.1674148745453121</v>
+        <v>-0.2953330102222519</v>
       </c>
       <c r="N9" t="n">
-        <v>-0.04267410516077448</v>
+        <v>-1.080290080349977</v>
       </c>
     </row>
     <row r="10">
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.2543932332295685</v>
+        <v>2.957712512974742</v>
       </c>
       <c r="D10" t="n">
-        <v>0.1321530467052584</v>
+        <v>0.8834826963492838</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -896,10 +896,10 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.2631341756960587</v>
+        <v>3.005683408205515</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1251788276899445</v>
+        <v>0.8951165367103356</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -912,10 +912,10 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>0.2594751685229012</v>
+        <v>2.971716986628217</v>
       </c>
       <c r="N10" t="n">
-        <v>0.12883809362615</v>
+        <v>0.9442786714535627</v>
       </c>
     </row>
     <row r="11">
@@ -930,10 +930,10 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>-0.02694496624959242</v>
+        <v>-0.9404595083043583</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.5654544943409103</v>
+        <v>-5.930910374526855</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>-0.02903935979540158</v>
+        <v>-0.8544864743186811</v>
       </c>
       <c r="I11" t="n">
-        <v>-0.5717060664457597</v>
+        <v>-6.033056354608223</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -962,10 +962,10 @@
         </is>
       </c>
       <c r="M11" t="n">
-        <v>-0.0239645529213874</v>
+        <v>-0.8134255027041549</v>
       </c>
       <c r="N11" t="n">
-        <v>-0.5668393441903627</v>
+        <v>-5.974145710399199</v>
       </c>
     </row>
     <row r="12">
@@ -980,10 +980,10 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.3384404651037688</v>
+        <v>1.581952720825654</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.03345109572644645</v>
+        <v>0.04668671505060182</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -996,10 +996,10 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0.3409525513811542</v>
+        <v>1.634821407766888</v>
       </c>
       <c r="I12" t="n">
-        <v>-0.03814799062550849</v>
+        <v>0.3568836814224776</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1012,10 +1012,10 @@
         </is>
       </c>
       <c r="M12" t="n">
-        <v>0.3407925680165666</v>
+        <v>1.616468052155855</v>
       </c>
       <c r="N12" t="n">
-        <v>-0.03743564356174371</v>
+        <v>0.2358887094726741</v>
       </c>
     </row>
     <row r="13">
@@ -1030,10 +1030,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.1906673018718444</v>
+        <v>-1.343531226442729</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1134572968524386</v>
+        <v>0.1483426712767074</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1046,10 +1046,10 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>-0.1837407186032225</v>
+        <v>-1.293100042420864</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1125209540450305</v>
+        <v>0.131336023076076</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1062,10 +1062,10 @@
         </is>
       </c>
       <c r="M13" t="n">
-        <v>-0.1875587003259248</v>
+        <v>-1.301904105568838</v>
       </c>
       <c r="N13" t="n">
-        <v>0.1118003180359624</v>
+        <v>0.1314839219778353</v>
       </c>
     </row>
     <row r="14">
@@ -1080,10 +1080,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.2297105914701</v>
+        <v>3.857008554606717</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.04346078974451351</v>
+        <v>-1.16437844792428</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1096,10 +1096,10 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.2290511269299839</v>
+        <v>3.944597982112051</v>
       </c>
       <c r="I14" t="n">
-        <v>-0.03724406774845081</v>
+        <v>-0.9904169541358941</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1112,10 +1112,10 @@
         </is>
       </c>
       <c r="M14" t="n">
-        <v>0.2348660580236924</v>
+        <v>3.952554849359154</v>
       </c>
       <c r="N14" t="n">
-        <v>-0.04551944114589217</v>
+        <v>-1.058729825538115</v>
       </c>
     </row>
     <row r="15">
@@ -1130,10 +1130,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-0.09226699501984105</v>
+        <v>-1.167781205230546</v>
       </c>
       <c r="D15" t="n">
-        <v>0.06594611365569769</v>
+        <v>0.06438230987133055</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -1146,10 +1146,10 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>-0.08760102009393134</v>
+        <v>-1.144668275285066</v>
       </c>
       <c r="I15" t="n">
-        <v>0.06664126621888654</v>
+        <v>0.007104247055822606</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1162,10 +1162,10 @@
         </is>
       </c>
       <c r="M15" t="n">
-        <v>-0.08914495518164411</v>
+        <v>-1.156619782799585</v>
       </c>
       <c r="N15" t="n">
-        <v>0.06400339890925587</v>
+        <v>0.0049806524848614</v>
       </c>
     </row>
     <row r="16">
@@ -1180,10 +1180,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.2037937483666964</v>
+        <v>1.010800030092929</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.2318380357701733</v>
+        <v>-1.009976785101278</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -1196,10 +1196,10 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.2025922520097224</v>
+        <v>1.074635358510046</v>
       </c>
       <c r="I16" t="n">
-        <v>-0.2309665414922339</v>
+        <v>-0.7771008870913128</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1212,10 +1212,10 @@
         </is>
       </c>
       <c r="M16" t="n">
-        <v>0.2047427785682162</v>
+        <v>1.062754267486645</v>
       </c>
       <c r="N16" t="n">
-        <v>-0.2346490339778434</v>
+        <v>-0.8796751785644247</v>
       </c>
     </row>
     <row r="17">
@@ -1230,10 +1230,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-0.402392482961469</v>
+        <v>-2.991341142456248</v>
       </c>
       <c r="D17" t="n">
-        <v>0.03029653509642153</v>
+        <v>1.255393055273236</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1246,10 +1246,10 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>-0.3973030544728168</v>
+        <v>-2.988799077626507</v>
       </c>
       <c r="I17" t="n">
-        <v>0.03351824361827578</v>
+        <v>1.075339638721587</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1262,10 +1262,10 @@
         </is>
       </c>
       <c r="M17" t="n">
-        <v>-0.3982782218148933</v>
+        <v>-3.002458865028825</v>
       </c>
       <c r="N17" t="n">
-        <v>0.02922050931212068</v>
+        <v>1.11710311423505</v>
       </c>
     </row>
     <row r="18">
@@ -1280,10 +1280,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.005300459464207453</v>
+        <v>-0.1831770216312719</v>
       </c>
       <c r="D18" t="n">
-        <v>0.01113383698636302</v>
+        <v>0.09290062701462738</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1296,10 +1296,10 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0.006406592386949202</v>
+        <v>-0.1595037252941525</v>
       </c>
       <c r="I18" t="n">
-        <v>0.0132331136682218</v>
+        <v>0.1260922149686351</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="M18" t="n">
-        <v>0.008524831313428427</v>
+        <v>-0.156537184126024</v>
       </c>
       <c r="N18" t="n">
-        <v>0.00876143205441513</v>
+        <v>0.1031566639250307</v>
       </c>
     </row>
     <row r="19">
@@ -1330,10 +1330,10 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.07367632616617667</v>
+        <v>0.3685054575778032</v>
       </c>
       <c r="D19" t="n">
-        <v>0.008711020552211799</v>
+        <v>0.1924378956679295</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1346,10 +1346,10 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>0.01982967251047285</v>
+        <v>-0.06612751791992247</v>
       </c>
       <c r="I19" t="n">
-        <v>0.008551532279022315</v>
+        <v>0.1439400408205036</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1362,10 +1362,60 @@
         </is>
       </c>
       <c r="M19" t="n">
-        <v>0.01330008778548898</v>
+        <v>0.1848993635689567</v>
       </c>
       <c r="N19" t="n">
-        <v>0.04618118473147973</v>
+        <v>0.08260740602562988</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>FL_recal</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0.05272373491571253</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.3641675324465929</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>FL_recal</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>-0.07675320573426836</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.1500417612960487</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>EN</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>FL_recal</t>
+        </is>
+      </c>
+      <c r="M20" t="n">
+        <v>-0.2530530976023811</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.3212421748219494</v>
       </c>
     </row>
     <row r="22">
@@ -1397,10 +1447,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.2466578442925881</v>
+        <v>3.785384654200639</v>
       </c>
       <c r="D23" t="n">
-        <v>0.3899444056915118</v>
+        <v>1.43129301980381</v>
       </c>
     </row>
     <row r="24">
@@ -1415,10 +1465,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.03909669504152156</v>
+        <v>-0.8658617014388169</v>
       </c>
       <c r="D24" t="n">
-        <v>-0.1015411505796034</v>
+        <v>-0.3862616280325226</v>
       </c>
     </row>
     <row r="25">
@@ -1433,10 +1483,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>-0.1366116352991686</v>
+        <v>-1.077390430003839</v>
       </c>
       <c r="D25" t="n">
-        <v>0.02286872659950226</v>
+        <v>-0.02368603403942836</v>
       </c>
     </row>
     <row r="26">
@@ -1451,10 +1501,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>-0.003807463327852231</v>
+        <v>-0.2738278321054153</v>
       </c>
       <c r="D26" t="n">
-        <v>-0.0121642297132783</v>
+        <v>-0.08987914134249703</v>
       </c>
     </row>
     <row r="27">
@@ -1469,10 +1519,10 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.135632447004005</v>
+        <v>-0.05164046799794583</v>
       </c>
       <c r="D27" t="n">
-        <v>0.01306803733519583</v>
+        <v>2.000146189747458</v>
       </c>
     </row>
     <row r="28">
@@ -1487,10 +1537,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>-0.4048869862639414</v>
+        <v>-3.699553146156773</v>
       </c>
       <c r="D28" t="n">
-        <v>0.0660995546155403</v>
+        <v>1.436360108198976</v>
       </c>
     </row>
     <row r="29">
@@ -1505,10 +1555,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>-0.06998848781086475</v>
+        <v>-0.583531765745646</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1803548057004144</v>
+        <v>1.715694547407411</v>
       </c>
     </row>
     <row r="30">
@@ -1523,10 +1573,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>-0.1703887698315676</v>
+        <v>-0.3098865152751313</v>
       </c>
       <c r="D30" t="n">
-        <v>-0.04021393053338585</v>
+        <v>-1.168914664933708</v>
       </c>
     </row>
     <row r="31">
@@ -1541,10 +1591,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.2631291658049845</v>
+        <v>3.005649312542155</v>
       </c>
       <c r="D31" t="n">
-        <v>0.1251949710621338</v>
+        <v>0.8951751011535413</v>
       </c>
     </row>
     <row r="32">
@@ -1559,10 +1609,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>-0.02901711910827857</v>
+        <v>-0.8543457718992837</v>
       </c>
       <c r="D32" t="n">
-        <v>-0.571703389385725</v>
+        <v>-6.033062612597332</v>
       </c>
     </row>
     <row r="33">
@@ -1577,10 +1627,10 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0.3409582568116613</v>
+        <v>1.634820173119677</v>
       </c>
       <c r="D33" t="n">
-        <v>-0.03813864643835112</v>
+        <v>0.3568651272311802</v>
       </c>
     </row>
     <row r="34">
@@ -1595,10 +1645,10 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>-0.1837515895010965</v>
+        <v>-1.293138331451671</v>
       </c>
       <c r="D34" t="n">
-        <v>0.1125141719452698</v>
+        <v>0.1313120642831169</v>
       </c>
     </row>
     <row r="35">
@@ -1613,10 +1663,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.2290639648404942</v>
+        <v>3.944640346511343</v>
       </c>
       <c r="D35" t="n">
-        <v>-0.03724106399154328</v>
+        <v>-0.9903911101493286</v>
       </c>
     </row>
     <row r="36">
@@ -1631,10 +1681,10 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>-0.08760742093602597</v>
+        <v>-1.144693738963819</v>
       </c>
       <c r="D36" t="n">
-        <v>0.06663663264833315</v>
+        <v>0.007071098718929719</v>
       </c>
     </row>
     <row r="37">
@@ -1649,10 +1699,10 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0.2026084335611877</v>
+        <v>1.074644874899488</v>
       </c>
       <c r="D37" t="n">
-        <v>-0.2309728764406564</v>
+        <v>-0.7770826925052322</v>
       </c>
     </row>
     <row r="38">
@@ -1667,10 +1717,10 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>-0.3973157453152085</v>
+        <v>-2.988787457679693</v>
       </c>
       <c r="D38" t="n">
-        <v>0.03351473672095836</v>
+        <v>1.075318744155036</v>
       </c>
     </row>
     <row r="39">
@@ -1685,10 +1735,10 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.006398439937418612</v>
+        <v>-0.1595865983894405</v>
       </c>
       <c r="D39" t="n">
-        <v>0.01322878019494396</v>
+        <v>0.1260729997154929</v>
       </c>
     </row>
     <row r="40">
@@ -1703,10 +1753,28 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.01982997010014317</v>
+        <v>-0.06613512379829439</v>
       </c>
       <c r="D40" t="n">
-        <v>0.008550464568740134</v>
+        <v>0.1439338282521111</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>noreg</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>FL_recal</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>-0.07676048036753093</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0.1500350549329869</v>
       </c>
     </row>
   </sheetData>

</xml_diff>